<commit_message>
update and fix some
separate rankings from conclusions sheet and use Friedman Test for ranking
</commit_message>
<xml_diff>
--- a/src/results_template/CEC2005/fixDim.xlsx
+++ b/src/results_template/CEC2005/fixDim.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\Research\Project Test\Base-Optimization-Framework\src\results_template\CEC2005\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\Research\Project Test\src\results_template\CEC2005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9643F0C-BA2F-4901-A43F-08EDA7E5FAF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B0EFA61-7D3A-432B-97F9-D6EF702C01C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conclusions" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="113">
   <si>
     <t>Comparison of optimization results for the CEC benchmark functions 2005 (Fix Dim)</t>
   </si>
@@ -176,132 +176,129 @@
     <t>F23</t>
   </si>
   <si>
-    <t>Number of Best Functions</t>
+    <t>P-value of the one-sided Welch t-test for the CEC benchmark functions 2005 (Fix Dim)</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>alg_base vs alg2</t>
+  </si>
+  <si>
+    <t>alg_base vs alg3</t>
+  </si>
+  <si>
+    <t>alg_base vs alg4</t>
+  </si>
+  <si>
+    <t>alg_base vs alg5</t>
+  </si>
+  <si>
+    <t>alg_base vs alg6</t>
+  </si>
+  <si>
+    <t>alg_base vs alg7</t>
+  </si>
+  <si>
+    <t>alg_base vs alg8</t>
+  </si>
+  <si>
+    <t>alg_base vs alg9</t>
+  </si>
+  <si>
+    <t>alg_base vs alg10</t>
+  </si>
+  <si>
+    <t>alg_base vs alg11</t>
+  </si>
+  <si>
+    <t>alg_base vs alg12</t>
+  </si>
+  <si>
+    <t>alg_base vs alg13</t>
+  </si>
+  <si>
+    <t>alg_base vs alg14</t>
+  </si>
+  <si>
+    <t>alg_base vs alg15</t>
+  </si>
+  <si>
+    <t>Decision (h) of the one-sided Welch t-test for the CEC benchmark functions 2005 (Fix Dim)</t>
+  </si>
+  <si>
+    <t>P-value of the one-sided Wilcoxon rank-sum test for the CEC benchmark functions 2005 (Fix Dim)</t>
+  </si>
+  <si>
+    <t>Decision (h) of the one-sided Wilcoxon rank-sum test for the CEC benchmark functions 2005 (Fix Dim)</t>
+  </si>
+  <si>
+    <t>Rank-sum statistic (W) for the Wilcoxon rank-sum test for the CEC benchmark functions 2005 (Fix Dim)</t>
+  </si>
+  <si>
+    <t>Function ranking and overall Friedman analysis for the CEC benchmark functions 2005 (Fix Dim)</t>
+  </si>
+  <si>
+    <t>Algorithm 1 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 2 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 3 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 4 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 5 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 6 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 7 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 8 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 9 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 10 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 11 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 12 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 13 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 14 Rank</t>
+  </si>
+  <si>
+    <t>Algorithm 15 Rank</t>
+  </si>
+  <si>
+    <t>Best Algorithm</t>
+  </si>
+  <si>
+    <t>Kruskal-Wallis p</t>
+  </si>
+  <si>
+    <t>Significant?</t>
+  </si>
+  <si>
+    <t>Average Rank</t>
   </si>
   <si>
     <t>Overall Rank</t>
   </si>
   <si>
-    <t>P-value of the one-sided Welch t-test for the CEC benchmark functions 2005 (Fix Dim)</t>
-  </si>
-  <si>
-    <t>Function</t>
-  </si>
-  <si>
-    <t>alg_base vs alg2</t>
-  </si>
-  <si>
-    <t>alg_base vs alg3</t>
-  </si>
-  <si>
-    <t>alg_base vs alg4</t>
-  </si>
-  <si>
-    <t>alg_base vs alg5</t>
-  </si>
-  <si>
-    <t>alg_base vs alg6</t>
-  </si>
-  <si>
-    <t>alg_base vs alg7</t>
-  </si>
-  <si>
-    <t>alg_base vs alg8</t>
-  </si>
-  <si>
-    <t>alg_base vs alg9</t>
-  </si>
-  <si>
-    <t>alg_base vs alg10</t>
-  </si>
-  <si>
-    <t>alg_base vs alg11</t>
-  </si>
-  <si>
-    <t>alg_base vs alg12</t>
-  </si>
-  <si>
-    <t>alg_base vs alg13</t>
-  </si>
-  <si>
-    <t>alg_base vs alg14</t>
-  </si>
-  <si>
-    <t>alg_base vs alg15</t>
-  </si>
-  <si>
-    <t>Decision (h) of the one-sided Welch t-test for the CEC benchmark functions 2005 (Fix Dim)</t>
-  </si>
-  <si>
-    <t>P-value of the one-sided Wilcoxon rank-sum test for the CEC benchmark functions 2005 (Fix Dim)</t>
-  </si>
-  <si>
-    <t>Decision (h) of the one-sided Wilcoxon rank-sum test for the CEC benchmark functions 2005 (Fix Dim)</t>
-  </si>
-  <si>
-    <t>Rank-sum statistic (W) for the Wilcoxon rank-sum test for the CEC benchmark functions 2005 (Fix Dim)</t>
-  </si>
-  <si>
-    <t>Function ranking and overall Friedman analysis for the CEC benchmark functions 2005 (Fix Dim)</t>
-  </si>
-  <si>
-    <t>Algorithm 1 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 2 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 3 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 4 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 5 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 6 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 7 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 8 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 9 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 10 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 11 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 12 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 13 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 14 Rank</t>
-  </si>
-  <si>
-    <t>Algorithm 15 Rank</t>
-  </si>
-  <si>
-    <t>Best Algorithm</t>
-  </si>
-  <si>
-    <t>Kruskal-Wallis p</t>
-  </si>
-  <si>
-    <t>Significant?</t>
-  </si>
-  <si>
-    <t>Average Rank</t>
-  </si>
-  <si>
     <t>Overall Friedman Test</t>
   </si>
   <si>
@@ -372,6 +369,12 @@
   </si>
   <si>
     <t>Optional figures showing the distribution of final objective values across independent runs for each function and algorithm.</t>
+  </si>
+  <si>
+    <t>Total number of best answers</t>
+  </si>
+  <si>
+    <t>Total number of equal-best answers</t>
   </si>
 </sst>
 </file>
@@ -404,7 +407,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -520,22 +523,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -601,17 +593,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="11" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -623,23 +611,39 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -864,9 +868,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1004,11 +1008,11 @@
       <c r="R1" s="29"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
       <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1055,11 +1059,11 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="32" t="s">
+    <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="38" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -1082,10 +1086,8 @@
       <c r="R3" s="3"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" s="33"/>
-      <c r="B4" s="14" t="s">
-        <v>18</v>
-      </c>
+      <c r="A4" s="31"/>
+      <c r="B4" s="39"/>
       <c r="C4" s="4" t="s">
         <v>20</v>
       </c>
@@ -1106,10 +1108,8 @@
       <c r="R4" s="9"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="33"/>
-      <c r="B5" s="6" t="s">
-        <v>18</v>
-      </c>
+      <c r="A5" s="31"/>
+      <c r="B5" s="40"/>
       <c r="C5" s="6" t="s">
         <v>21</v>
       </c>
@@ -1130,8 +1130,8 @@
       <c r="R5" s="7"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="33"/>
-      <c r="B6" s="2" t="s">
+      <c r="A6" s="31"/>
+      <c r="B6" s="38" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="2" t="s">
@@ -1154,10 +1154,8 @@
       <c r="R6" s="3"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" s="33"/>
-      <c r="B7" s="14" t="s">
-        <v>22</v>
-      </c>
+      <c r="A7" s="31"/>
+      <c r="B7" s="39"/>
       <c r="C7" s="4" t="s">
         <v>20</v>
       </c>
@@ -1178,10 +1176,8 @@
       <c r="R7" s="9"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" s="33"/>
-      <c r="B8" s="6" t="s">
-        <v>22</v>
-      </c>
+      <c r="A8" s="31"/>
+      <c r="B8" s="40"/>
       <c r="C8" s="6" t="s">
         <v>21</v>
       </c>
@@ -1202,8 +1198,8 @@
       <c r="R8" s="7"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" s="33"/>
-      <c r="B9" s="2" t="s">
+      <c r="A9" s="31"/>
+      <c r="B9" s="38" t="s">
         <v>23</v>
       </c>
       <c r="C9" s="2" t="s">
@@ -1226,10 +1222,8 @@
       <c r="R9" s="3"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A10" s="33"/>
-      <c r="B10" s="14" t="s">
-        <v>23</v>
-      </c>
+      <c r="A10" s="31"/>
+      <c r="B10" s="39"/>
       <c r="C10" s="4" t="s">
         <v>20</v>
       </c>
@@ -1250,10 +1244,8 @@
       <c r="R10" s="9"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" s="33"/>
-      <c r="B11" s="6" t="s">
-        <v>23</v>
-      </c>
+      <c r="A11" s="31"/>
+      <c r="B11" s="40"/>
       <c r="C11" s="6" t="s">
         <v>21</v>
       </c>
@@ -1274,8 +1266,8 @@
       <c r="R11" s="7"/>
     </row>
     <row r="12" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="33"/>
-      <c r="B12" s="2" t="s">
+      <c r="A12" s="31"/>
+      <c r="B12" s="38" t="s">
         <v>24</v>
       </c>
       <c r="C12" s="2" t="s">
@@ -1298,10 +1290,8 @@
       <c r="R12" s="3"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A13" s="33"/>
-      <c r="B13" s="14" t="s">
-        <v>24</v>
-      </c>
+      <c r="A13" s="31"/>
+      <c r="B13" s="39"/>
       <c r="C13" s="4" t="s">
         <v>20</v>
       </c>
@@ -1322,10 +1312,8 @@
       <c r="R13" s="9"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A14" s="33"/>
-      <c r="B14" s="6" t="s">
-        <v>24</v>
-      </c>
+      <c r="A14" s="31"/>
+      <c r="B14" s="40"/>
       <c r="C14" s="6" t="s">
         <v>21</v>
       </c>
@@ -1346,8 +1334,8 @@
       <c r="R14" s="7"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A15" s="33"/>
-      <c r="B15" s="2" t="s">
+      <c r="A15" s="31"/>
+      <c r="B15" s="38" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="2" t="s">
@@ -1370,10 +1358,8 @@
       <c r="R15" s="3"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A16" s="33"/>
-      <c r="B16" s="14" t="s">
-        <v>25</v>
-      </c>
+      <c r="A16" s="31"/>
+      <c r="B16" s="39"/>
       <c r="C16" s="4" t="s">
         <v>20</v>
       </c>
@@ -1394,10 +1380,8 @@
       <c r="R16" s="9"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A17" s="33"/>
-      <c r="B17" s="6" t="s">
-        <v>25</v>
-      </c>
+      <c r="A17" s="31"/>
+      <c r="B17" s="40"/>
       <c r="C17" s="6" t="s">
         <v>21</v>
       </c>
@@ -1418,8 +1402,8 @@
       <c r="R17" s="7"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A18" s="33"/>
-      <c r="B18" s="2" t="s">
+      <c r="A18" s="31"/>
+      <c r="B18" s="38" t="s">
         <v>26</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1442,10 +1426,8 @@
       <c r="R18" s="3"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="33"/>
-      <c r="B19" s="14" t="s">
-        <v>26</v>
-      </c>
+      <c r="A19" s="31"/>
+      <c r="B19" s="39"/>
       <c r="C19" s="4" t="s">
         <v>20</v>
       </c>
@@ -1466,10 +1448,8 @@
       <c r="R19" s="9"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A20" s="33"/>
-      <c r="B20" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="A20" s="31"/>
+      <c r="B20" s="40"/>
       <c r="C20" s="6" t="s">
         <v>21</v>
       </c>
@@ -1490,8 +1470,8 @@
       <c r="R20" s="7"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A21" s="33"/>
-      <c r="B21" s="2" t="s">
+      <c r="A21" s="31"/>
+      <c r="B21" s="38" t="s">
         <v>27</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -1514,10 +1494,8 @@
       <c r="R21" s="3"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A22" s="33"/>
-      <c r="B22" s="14" t="s">
-        <v>27</v>
-      </c>
+      <c r="A22" s="31"/>
+      <c r="B22" s="39"/>
       <c r="C22" s="4" t="s">
         <v>20</v>
       </c>
@@ -1538,10 +1516,8 @@
       <c r="R22" s="9"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23" s="34"/>
-      <c r="B23" s="6" t="s">
-        <v>27</v>
-      </c>
+      <c r="A23" s="32"/>
+      <c r="B23" s="40"/>
       <c r="C23" s="6" t="s">
         <v>21</v>
       </c>
@@ -1562,10 +1538,10 @@
       <c r="R23" s="7"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A24" s="32" t="s">
+      <c r="A24" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="38" t="s">
         <v>29</v>
       </c>
       <c r="C24" s="2" t="s">
@@ -1588,10 +1564,8 @@
       <c r="R24" s="3"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A25" s="33"/>
-      <c r="B25" s="14" t="s">
-        <v>29</v>
-      </c>
+      <c r="A25" s="31"/>
+      <c r="B25" s="39"/>
       <c r="C25" s="4" t="s">
         <v>20</v>
       </c>
@@ -1612,10 +1586,8 @@
       <c r="R25" s="9"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A26" s="33"/>
-      <c r="B26" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="A26" s="31"/>
+      <c r="B26" s="40"/>
       <c r="C26" s="6" t="s">
         <v>21</v>
       </c>
@@ -1636,8 +1608,8 @@
       <c r="R26" s="7"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A27" s="33"/>
-      <c r="B27" s="2" t="s">
+      <c r="A27" s="31"/>
+      <c r="B27" s="38" t="s">
         <v>30</v>
       </c>
       <c r="C27" s="2" t="s">
@@ -1660,10 +1632,8 @@
       <c r="R27" s="3"/>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A28" s="33"/>
-      <c r="B28" s="14" t="s">
-        <v>30</v>
-      </c>
+      <c r="A28" s="31"/>
+      <c r="B28" s="39"/>
       <c r="C28" s="4" t="s">
         <v>20</v>
       </c>
@@ -1684,10 +1654,8 @@
       <c r="R28" s="9"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A29" s="33"/>
-      <c r="B29" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="A29" s="31"/>
+      <c r="B29" s="40"/>
       <c r="C29" s="6" t="s">
         <v>21</v>
       </c>
@@ -1708,8 +1676,8 @@
       <c r="R29" s="7"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A30" s="33"/>
-      <c r="B30" s="2" t="s">
+      <c r="A30" s="31"/>
+      <c r="B30" s="38" t="s">
         <v>31</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -1732,10 +1700,8 @@
       <c r="R30" s="3"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A31" s="33"/>
-      <c r="B31" s="14" t="s">
-        <v>31</v>
-      </c>
+      <c r="A31" s="31"/>
+      <c r="B31" s="39"/>
       <c r="C31" s="4" t="s">
         <v>20</v>
       </c>
@@ -1756,10 +1722,8 @@
       <c r="R31" s="9"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A32" s="33"/>
-      <c r="B32" s="6" t="s">
-        <v>31</v>
-      </c>
+      <c r="A32" s="31"/>
+      <c r="B32" s="40"/>
       <c r="C32" s="6" t="s">
         <v>21</v>
       </c>
@@ -1780,8 +1744,8 @@
       <c r="R32" s="7"/>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A33" s="33"/>
-      <c r="B33" s="2" t="s">
+      <c r="A33" s="31"/>
+      <c r="B33" s="38" t="s">
         <v>32</v>
       </c>
       <c r="C33" s="2" t="s">
@@ -1804,10 +1768,8 @@
       <c r="R33" s="3"/>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A34" s="33"/>
-      <c r="B34" s="14" t="s">
-        <v>32</v>
-      </c>
+      <c r="A34" s="31"/>
+      <c r="B34" s="39"/>
       <c r="C34" s="4" t="s">
         <v>20</v>
       </c>
@@ -1828,10 +1790,8 @@
       <c r="R34" s="9"/>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A35" s="33"/>
-      <c r="B35" s="6" t="s">
-        <v>32</v>
-      </c>
+      <c r="A35" s="31"/>
+      <c r="B35" s="40"/>
       <c r="C35" s="6" t="s">
         <v>21</v>
       </c>
@@ -1852,8 +1812,8 @@
       <c r="R35" s="7"/>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A36" s="33"/>
-      <c r="B36" s="2" t="s">
+      <c r="A36" s="31"/>
+      <c r="B36" s="38" t="s">
         <v>33</v>
       </c>
       <c r="C36" s="2" t="s">
@@ -1876,10 +1836,8 @@
       <c r="R36" s="3"/>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A37" s="33"/>
-      <c r="B37" s="14" t="s">
-        <v>33</v>
-      </c>
+      <c r="A37" s="31"/>
+      <c r="B37" s="39"/>
       <c r="C37" s="4" t="s">
         <v>20</v>
       </c>
@@ -1900,10 +1858,8 @@
       <c r="R37" s="9"/>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A38" s="33"/>
-      <c r="B38" s="6" t="s">
-        <v>33</v>
-      </c>
+      <c r="A38" s="31"/>
+      <c r="B38" s="40"/>
       <c r="C38" s="6" t="s">
         <v>21</v>
       </c>
@@ -1924,8 +1880,8 @@
       <c r="R38" s="7"/>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A39" s="33"/>
-      <c r="B39" s="2" t="s">
+      <c r="A39" s="31"/>
+      <c r="B39" s="38" t="s">
         <v>34</v>
       </c>
       <c r="C39" s="2" t="s">
@@ -1948,10 +1904,8 @@
       <c r="R39" s="3"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A40" s="33"/>
-      <c r="B40" s="14" t="s">
-        <v>34</v>
-      </c>
+      <c r="A40" s="31"/>
+      <c r="B40" s="39"/>
       <c r="C40" s="4" t="s">
         <v>20</v>
       </c>
@@ -1972,10 +1926,8 @@
       <c r="R40" s="9"/>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A41" s="33"/>
-      <c r="B41" s="6" t="s">
-        <v>34</v>
-      </c>
+      <c r="A41" s="31"/>
+      <c r="B41" s="40"/>
       <c r="C41" s="6" t="s">
         <v>21</v>
       </c>
@@ -1996,8 +1948,8 @@
       <c r="R41" s="7"/>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A42" s="33"/>
-      <c r="B42" s="2" t="s">
+      <c r="A42" s="31"/>
+      <c r="B42" s="38" t="s">
         <v>35</v>
       </c>
       <c r="C42" s="2" t="s">
@@ -2020,10 +1972,8 @@
       <c r="R42" s="3"/>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A43" s="33"/>
-      <c r="B43" s="14" t="s">
-        <v>35</v>
-      </c>
+      <c r="A43" s="31"/>
+      <c r="B43" s="39"/>
       <c r="C43" s="4" t="s">
         <v>20</v>
       </c>
@@ -2044,10 +1994,8 @@
       <c r="R43" s="9"/>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A44" s="33"/>
-      <c r="B44" s="6" t="s">
-        <v>35</v>
-      </c>
+      <c r="A44" s="31"/>
+      <c r="B44" s="40"/>
       <c r="C44" s="6" t="s">
         <v>21</v>
       </c>
@@ -2068,8 +2016,8 @@
       <c r="R44" s="7"/>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A45" s="33"/>
-      <c r="B45" s="2" t="s">
+      <c r="A45" s="31"/>
+      <c r="B45" s="38" t="s">
         <v>36</v>
       </c>
       <c r="C45" s="2" t="s">
@@ -2092,10 +2040,8 @@
       <c r="R45" s="3"/>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A46" s="33"/>
-      <c r="B46" s="14" t="s">
-        <v>36</v>
-      </c>
+      <c r="A46" s="31"/>
+      <c r="B46" s="39"/>
       <c r="C46" s="4" t="s">
         <v>20</v>
       </c>
@@ -2116,10 +2062,8 @@
       <c r="R46" s="9"/>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A47" s="33"/>
-      <c r="B47" s="6" t="s">
-        <v>36</v>
-      </c>
+      <c r="A47" s="31"/>
+      <c r="B47" s="40"/>
       <c r="C47" s="6" t="s">
         <v>21</v>
       </c>
@@ -2140,8 +2084,8 @@
       <c r="R47" s="7"/>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A48" s="33"/>
-      <c r="B48" s="2" t="s">
+      <c r="A48" s="31"/>
+      <c r="B48" s="38" t="s">
         <v>37</v>
       </c>
       <c r="C48" s="2" t="s">
@@ -2164,10 +2108,8 @@
       <c r="R48" s="3"/>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A49" s="33"/>
-      <c r="B49" s="14" t="s">
-        <v>37</v>
-      </c>
+      <c r="A49" s="31"/>
+      <c r="B49" s="39"/>
       <c r="C49" s="4" t="s">
         <v>20</v>
       </c>
@@ -2188,10 +2130,8 @@
       <c r="R49" s="9"/>
     </row>
     <row r="50" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A50" s="34"/>
-      <c r="B50" s="6" t="s">
-        <v>37</v>
-      </c>
+      <c r="A50" s="32"/>
+      <c r="B50" s="40"/>
       <c r="C50" s="6" t="s">
         <v>21</v>
       </c>
@@ -2212,10 +2152,10 @@
       <c r="R50" s="7"/>
     </row>
     <row r="51" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="32" t="s">
+      <c r="A51" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="2" t="s">
+      <c r="B51" s="38" t="s">
         <v>39</v>
       </c>
       <c r="C51" s="2" t="s">
@@ -2238,10 +2178,8 @@
       <c r="R51" s="3"/>
     </row>
     <row r="52" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A52" s="33"/>
-      <c r="B52" s="14" t="s">
-        <v>39</v>
-      </c>
+      <c r="A52" s="31"/>
+      <c r="B52" s="39"/>
       <c r="C52" s="4" t="s">
         <v>20</v>
       </c>
@@ -2262,10 +2200,8 @@
       <c r="R52" s="9"/>
     </row>
     <row r="53" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A53" s="33"/>
-      <c r="B53" s="6" t="s">
-        <v>39</v>
-      </c>
+      <c r="A53" s="31"/>
+      <c r="B53" s="40"/>
       <c r="C53" s="6" t="s">
         <v>21</v>
       </c>
@@ -2286,8 +2222,8 @@
       <c r="R53" s="7"/>
     </row>
     <row r="54" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A54" s="33"/>
-      <c r="B54" s="2" t="s">
+      <c r="A54" s="31"/>
+      <c r="B54" s="38" t="s">
         <v>40</v>
       </c>
       <c r="C54" s="2" t="s">
@@ -2310,10 +2246,8 @@
       <c r="R54" s="3"/>
     </row>
     <row r="55" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A55" s="33"/>
-      <c r="B55" s="14" t="s">
-        <v>40</v>
-      </c>
+      <c r="A55" s="31"/>
+      <c r="B55" s="39"/>
       <c r="C55" s="4" t="s">
         <v>20</v>
       </c>
@@ -2334,10 +2268,8 @@
       <c r="R55" s="9"/>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A56" s="33"/>
-      <c r="B56" s="6" t="s">
-        <v>40</v>
-      </c>
+      <c r="A56" s="31"/>
+      <c r="B56" s="40"/>
       <c r="C56" s="6" t="s">
         <v>21</v>
       </c>
@@ -2358,8 +2290,8 @@
       <c r="R56" s="7"/>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A57" s="33"/>
-      <c r="B57" s="2" t="s">
+      <c r="A57" s="31"/>
+      <c r="B57" s="38" t="s">
         <v>41</v>
       </c>
       <c r="C57" s="2" t="s">
@@ -2382,10 +2314,8 @@
       <c r="R57" s="3"/>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A58" s="33"/>
-      <c r="B58" s="14" t="s">
-        <v>41</v>
-      </c>
+      <c r="A58" s="31"/>
+      <c r="B58" s="39"/>
       <c r="C58" s="4" t="s">
         <v>20</v>
       </c>
@@ -2406,10 +2336,8 @@
       <c r="R58" s="9"/>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A59" s="33"/>
-      <c r="B59" s="6" t="s">
-        <v>41</v>
-      </c>
+      <c r="A59" s="31"/>
+      <c r="B59" s="40"/>
       <c r="C59" s="6" t="s">
         <v>21</v>
       </c>
@@ -2430,8 +2358,8 @@
       <c r="R59" s="7"/>
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A60" s="33"/>
-      <c r="B60" s="2" t="s">
+      <c r="A60" s="31"/>
+      <c r="B60" s="38" t="s">
         <v>42</v>
       </c>
       <c r="C60" s="2" t="s">
@@ -2454,10 +2382,8 @@
       <c r="R60" s="3"/>
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A61" s="33"/>
-      <c r="B61" s="14" t="s">
-        <v>42</v>
-      </c>
+      <c r="A61" s="31"/>
+      <c r="B61" s="39"/>
       <c r="C61" s="4" t="s">
         <v>20</v>
       </c>
@@ -2478,10 +2404,8 @@
       <c r="R61" s="9"/>
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A62" s="33"/>
-      <c r="B62" s="6" t="s">
-        <v>42</v>
-      </c>
+      <c r="A62" s="31"/>
+      <c r="B62" s="40"/>
       <c r="C62" s="6" t="s">
         <v>21</v>
       </c>
@@ -2502,8 +2426,8 @@
       <c r="R62" s="7"/>
     </row>
     <row r="63" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A63" s="33"/>
-      <c r="B63" s="2" t="s">
+      <c r="A63" s="31"/>
+      <c r="B63" s="38" t="s">
         <v>43</v>
       </c>
       <c r="C63" s="2" t="s">
@@ -2526,10 +2450,8 @@
       <c r="R63" s="3"/>
     </row>
     <row r="64" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A64" s="33"/>
-      <c r="B64" s="14" t="s">
-        <v>43</v>
-      </c>
+      <c r="A64" s="31"/>
+      <c r="B64" s="39"/>
       <c r="C64" s="4" t="s">
         <v>20</v>
       </c>
@@ -2550,10 +2472,8 @@
       <c r="R64" s="9"/>
     </row>
     <row r="65" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A65" s="33"/>
-      <c r="B65" s="6" t="s">
-        <v>43</v>
-      </c>
+      <c r="A65" s="31"/>
+      <c r="B65" s="40"/>
       <c r="C65" s="6" t="s">
         <v>21</v>
       </c>
@@ -2574,8 +2494,8 @@
       <c r="R65" s="7"/>
     </row>
     <row r="66" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A66" s="33"/>
-      <c r="B66" s="2" t="s">
+      <c r="A66" s="31"/>
+      <c r="B66" s="38" t="s">
         <v>44</v>
       </c>
       <c r="C66" s="2" t="s">
@@ -2598,10 +2518,8 @@
       <c r="R66" s="3"/>
     </row>
     <row r="67" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A67" s="33"/>
-      <c r="B67" s="14" t="s">
-        <v>44</v>
-      </c>
+      <c r="A67" s="31"/>
+      <c r="B67" s="39"/>
       <c r="C67" s="4" t="s">
         <v>20</v>
       </c>
@@ -2622,10 +2540,8 @@
       <c r="R67" s="9"/>
     </row>
     <row r="68" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A68" s="33"/>
-      <c r="B68" s="6" t="s">
-        <v>44</v>
-      </c>
+      <c r="A68" s="31"/>
+      <c r="B68" s="40"/>
       <c r="C68" s="6" t="s">
         <v>21</v>
       </c>
@@ -2646,8 +2562,8 @@
       <c r="R68" s="7"/>
     </row>
     <row r="69" spans="1:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="33"/>
-      <c r="B69" s="2" t="s">
+      <c r="A69" s="31"/>
+      <c r="B69" s="38" t="s">
         <v>45</v>
       </c>
       <c r="C69" s="2" t="s">
@@ -2670,10 +2586,8 @@
       <c r="R69" s="3"/>
     </row>
     <row r="70" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A70" s="33"/>
-      <c r="B70" s="14" t="s">
-        <v>45</v>
-      </c>
+      <c r="A70" s="31"/>
+      <c r="B70" s="39"/>
       <c r="C70" s="4" t="s">
         <v>20</v>
       </c>
@@ -2694,10 +2608,8 @@
       <c r="R70" s="9"/>
     </row>
     <row r="71" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A71" s="34"/>
-      <c r="B71" s="6" t="s">
-        <v>45</v>
-      </c>
+      <c r="A71" s="32"/>
+      <c r="B71" s="40"/>
       <c r="C71" s="6" t="s">
         <v>21</v>
       </c>
@@ -2718,43 +2630,66 @@
       <c r="R71" s="7"/>
     </row>
     <row r="72" spans="1:18" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="32" t="s">
-        <v>46</v>
-      </c>
-      <c r="B72" s="35"/>
-      <c r="C72" s="35"/>
+      <c r="A72" s="33" t="s">
+        <v>111</v>
+      </c>
+      <c r="B72" s="34"/>
+      <c r="C72" s="34"/>
     </row>
     <row r="73" spans="1:18" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="30" t="s">
-        <v>47</v>
-      </c>
-      <c r="B73" s="31"/>
-      <c r="C73" s="31"/>
-      <c r="D73" s="27"/>
-      <c r="E73" s="27"/>
-      <c r="F73" s="27"/>
-      <c r="G73" s="27"/>
-      <c r="H73" s="27"/>
-      <c r="I73" s="27"/>
-      <c r="J73" s="27"/>
-      <c r="K73" s="27"/>
-      <c r="L73" s="27"/>
-      <c r="M73" s="27"/>
-      <c r="N73" s="27"/>
-      <c r="O73" s="27"/>
-      <c r="P73" s="27"/>
-      <c r="Q73" s="27"/>
-      <c r="R73" s="27"/>
+      <c r="A73" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="B73" s="37"/>
+      <c r="C73" s="37"/>
+      <c r="D73" s="28"/>
+      <c r="E73" s="28"/>
+      <c r="F73" s="28"/>
+      <c r="G73" s="28"/>
+      <c r="H73" s="28"/>
+      <c r="I73" s="28"/>
+      <c r="J73" s="28"/>
+      <c r="K73" s="28"/>
+      <c r="L73" s="28"/>
+      <c r="M73" s="28"/>
+      <c r="N73" s="28"/>
+      <c r="O73" s="28"/>
+      <c r="P73" s="28"/>
+      <c r="Q73" s="28"/>
+      <c r="R73" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="30">
+    <mergeCell ref="A73:C73"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="B45:B47"/>
     <mergeCell ref="A1:R1"/>
-    <mergeCell ref="A73:C73"/>
     <mergeCell ref="A3:A23"/>
     <mergeCell ref="A24:A50"/>
     <mergeCell ref="A51:A71"/>
     <mergeCell ref="A72:C72"/>
     <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="B54:B56"/>
+    <mergeCell ref="B57:B59"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="B63:B65"/>
+    <mergeCell ref="B66:B68"/>
+    <mergeCell ref="B69:B71"/>
   </mergeCells>
   <conditionalFormatting sqref="D3:R3">
     <cfRule type="top10" dxfId="26" priority="31" bottom="1" rank="1"/>
@@ -2840,69 +2775,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="A1" s="41" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="D2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="E2" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="F2" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="G2" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="H2" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="I2" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="J2" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="K2" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="L2" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="M2" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="N2" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="O2" s="18" t="s">
         <v>61</v>
-      </c>
-      <c r="N2" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -3367,69 +3302,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
-        <v>64</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="A1" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="D2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="E2" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="F2" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="G2" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="H2" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="I2" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="J2" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="K2" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="L2" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="M2" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="N2" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="O2" s="18" t="s">
         <v>61</v>
-      </c>
-      <c r="N2" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -3893,69 +3828,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
-        <v>65</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="A1" s="41" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="D2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="E2" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="F2" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="G2" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="H2" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="I2" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="J2" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="K2" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="L2" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="M2" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="N2" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="O2" s="18" t="s">
         <v>61</v>
-      </c>
-      <c r="N2" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -4420,69 +4355,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
-        <v>66</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="A1" s="41" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="D2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="E2" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="F2" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="G2" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="H2" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="I2" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="J2" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="K2" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="L2" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="M2" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="N2" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="O2" s="18" t="s">
         <v>61</v>
-      </c>
-      <c r="N2" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -4947,69 +4882,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
-        <v>67</v>
-      </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
+      <c r="A1" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
+      <c r="M1" s="41"/>
+      <c r="N1" s="41"/>
+      <c r="O1" s="41"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="D2" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="E2" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="F2" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="G2" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="H2" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="I2" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="J2" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="K2" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="L2" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="M2" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="N2" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="O2" s="18" t="s">
         <v>61</v>
-      </c>
-      <c r="N2" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="O2" s="18" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -5154,115 +5089,116 @@
   <dimension ref="A1:S40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="10" width="16.140625" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="10" width="16.140625" customWidth="1"/>
     <col min="11" max="16" width="17.28515625" customWidth="1"/>
-    <col min="17" max="17" width="20" customWidth="1"/>
-    <col min="18" max="18" width="18" customWidth="1"/>
-    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="17" max="17" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="44" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="S1" s="44"/>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="43" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="43" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="43" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-      <c r="L1" s="38"/>
-      <c r="M1" s="38"/>
-      <c r="N1" s="38"/>
-      <c r="O1" s="38"/>
-      <c r="P1" s="38"/>
-      <c r="Q1" s="38"/>
-      <c r="R1" s="38"/>
-      <c r="S1" s="38"/>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" s="28" t="s">
+      <c r="D2" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="E2" s="43" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="F2" s="43" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="G2" s="43" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="H2" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="G2" s="28" t="s">
+      <c r="I2" s="43" t="s">
         <v>74</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="J2" s="43" t="s">
         <v>75</v>
       </c>
-      <c r="I2" s="28" t="s">
+      <c r="K2" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="J2" s="28" t="s">
+      <c r="L2" s="43" t="s">
         <v>77</v>
       </c>
-      <c r="K2" s="28" t="s">
+      <c r="M2" s="43" t="s">
         <v>78</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="N2" s="43" t="s">
         <v>79</v>
       </c>
-      <c r="M2" s="28" t="s">
+      <c r="O2" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="N2" s="28" t="s">
+      <c r="P2" s="43" t="s">
         <v>81</v>
       </c>
-      <c r="O2" s="28" t="s">
+      <c r="Q2" s="43" t="s">
         <v>82</v>
       </c>
-      <c r="P2" s="28" t="s">
+      <c r="R2" s="43" t="s">
         <v>83</v>
       </c>
-      <c r="Q2" s="28" t="s">
+      <c r="S2" s="43" t="s">
         <v>84</v>
-      </c>
-      <c r="R2" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="S2" s="28" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="27"/>
+      <c r="N3" s="27"/>
+      <c r="O3" s="27"/>
+      <c r="P3" s="27"/>
       <c r="Q3" s="19"/>
       <c r="R3" s="19"/>
       <c r="S3" s="19"/>
@@ -5271,21 +5207,21 @@
       <c r="A4" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="40"/>
-      <c r="K4" s="40"/>
-      <c r="L4" s="40"/>
-      <c r="M4" s="40"/>
-      <c r="N4" s="40"/>
-      <c r="O4" s="40"/>
-      <c r="P4" s="40"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="27"/>
+      <c r="K4" s="27"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
       <c r="Q4" s="19"/>
       <c r="R4" s="19"/>
       <c r="S4" s="19"/>
@@ -5294,21 +5230,21 @@
       <c r="A5" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="40"/>
-      <c r="I5" s="40"/>
-      <c r="J5" s="40"/>
-      <c r="K5" s="40"/>
-      <c r="L5" s="40"/>
-      <c r="M5" s="40"/>
-      <c r="N5" s="40"/>
-      <c r="O5" s="40"/>
-      <c r="P5" s="40"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="27"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="27"/>
+      <c r="P5" s="27"/>
       <c r="Q5" s="19"/>
       <c r="R5" s="19"/>
       <c r="S5" s="19"/>
@@ -5317,21 +5253,21 @@
       <c r="A6" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="40"/>
-      <c r="J6" s="40"/>
-      <c r="K6" s="40"/>
-      <c r="L6" s="40"/>
-      <c r="M6" s="40"/>
-      <c r="N6" s="40"/>
-      <c r="O6" s="40"/>
-      <c r="P6" s="40"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="27"/>
+      <c r="M6" s="27"/>
+      <c r="N6" s="27"/>
+      <c r="O6" s="27"/>
+      <c r="P6" s="27"/>
       <c r="Q6" s="19"/>
       <c r="R6" s="19"/>
       <c r="S6" s="19"/>
@@ -5340,21 +5276,21 @@
       <c r="A7" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
-      <c r="G7" s="40"/>
-      <c r="H7" s="40"/>
-      <c r="I7" s="40"/>
-      <c r="J7" s="40"/>
-      <c r="K7" s="40"/>
-      <c r="L7" s="40"/>
-      <c r="M7" s="40"/>
-      <c r="N7" s="40"/>
-      <c r="O7" s="40"/>
-      <c r="P7" s="40"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
+      <c r="K7" s="27"/>
+      <c r="L7" s="27"/>
+      <c r="M7" s="27"/>
+      <c r="N7" s="27"/>
+      <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
       <c r="Q7" s="19"/>
       <c r="R7" s="19"/>
       <c r="S7" s="19"/>
@@ -5363,21 +5299,21 @@
       <c r="A8" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="40"/>
-      <c r="K8" s="40"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="40"/>
-      <c r="N8" s="40"/>
-      <c r="O8" s="40"/>
-      <c r="P8" s="40"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="27"/>
+      <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
       <c r="Q8" s="19"/>
       <c r="R8" s="19"/>
       <c r="S8" s="19"/>
@@ -5386,21 +5322,21 @@
       <c r="A9" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="40"/>
-      <c r="C9" s="40"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="40"/>
-      <c r="F9" s="40"/>
-      <c r="G9" s="40"/>
-      <c r="H9" s="40"/>
-      <c r="I9" s="40"/>
-      <c r="J9" s="40"/>
-      <c r="K9" s="40"/>
-      <c r="L9" s="40"/>
-      <c r="M9" s="40"/>
-      <c r="N9" s="40"/>
-      <c r="O9" s="40"/>
-      <c r="P9" s="40"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
+      <c r="K9" s="27"/>
+      <c r="L9" s="27"/>
+      <c r="M9" s="27"/>
+      <c r="N9" s="27"/>
+      <c r="O9" s="27"/>
+      <c r="P9" s="27"/>
       <c r="Q9" s="19"/>
       <c r="R9" s="19"/>
       <c r="S9" s="19"/>
@@ -5409,21 +5345,21 @@
       <c r="A10" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="40"/>
-      <c r="C10" s="40"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="40"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="40"/>
-      <c r="K10" s="40"/>
-      <c r="L10" s="40"/>
-      <c r="M10" s="40"/>
-      <c r="N10" s="40"/>
-      <c r="O10" s="40"/>
-      <c r="P10" s="40"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
+      <c r="L10" s="27"/>
+      <c r="M10" s="27"/>
+      <c r="N10" s="27"/>
+      <c r="O10" s="27"/>
+      <c r="P10" s="27"/>
       <c r="Q10" s="19"/>
       <c r="R10" s="19"/>
       <c r="S10" s="19"/>
@@ -5432,21 +5368,21 @@
       <c r="A11" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="40"/>
-      <c r="C11" s="40"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="40"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="40"/>
-      <c r="J11" s="40"/>
-      <c r="K11" s="40"/>
-      <c r="L11" s="40"/>
-      <c r="M11" s="40"/>
-      <c r="N11" s="40"/>
-      <c r="O11" s="40"/>
-      <c r="P11" s="40"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
+      <c r="K11" s="27"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="27"/>
+      <c r="P11" s="27"/>
       <c r="Q11" s="19"/>
       <c r="R11" s="19"/>
       <c r="S11" s="19"/>
@@ -5455,21 +5391,21 @@
       <c r="A12" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="40"/>
-      <c r="J12" s="40"/>
-      <c r="K12" s="40"/>
-      <c r="L12" s="40"/>
-      <c r="M12" s="40"/>
-      <c r="N12" s="40"/>
-      <c r="O12" s="40"/>
-      <c r="P12" s="40"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+      <c r="O12" s="27"/>
+      <c r="P12" s="27"/>
       <c r="Q12" s="19"/>
       <c r="R12" s="19"/>
       <c r="S12" s="19"/>
@@ -5478,21 +5414,21 @@
       <c r="A13" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="40"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="40"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="40"/>
-      <c r="J13" s="40"/>
-      <c r="K13" s="40"/>
-      <c r="L13" s="40"/>
-      <c r="M13" s="40"/>
-      <c r="N13" s="40"/>
-      <c r="O13" s="40"/>
-      <c r="P13" s="40"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
+      <c r="K13" s="27"/>
+      <c r="L13" s="27"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="27"/>
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
       <c r="Q13" s="19"/>
       <c r="R13" s="19"/>
       <c r="S13" s="19"/>
@@ -5501,21 +5437,21 @@
       <c r="A14" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="40"/>
-      <c r="C14" s="40"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="40"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="40"/>
-      <c r="J14" s="40"/>
-      <c r="K14" s="40"/>
-      <c r="L14" s="40"/>
-      <c r="M14" s="40"/>
-      <c r="N14" s="40"/>
-      <c r="O14" s="40"/>
-      <c r="P14" s="40"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
+      <c r="L14" s="27"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="27"/>
+      <c r="O14" s="27"/>
+      <c r="P14" s="27"/>
       <c r="Q14" s="19"/>
       <c r="R14" s="19"/>
       <c r="S14" s="19"/>
@@ -5524,21 +5460,21 @@
       <c r="A15" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="B15" s="40"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="40"/>
-      <c r="K15" s="40"/>
-      <c r="L15" s="40"/>
-      <c r="M15" s="40"/>
-      <c r="N15" s="40"/>
-      <c r="O15" s="40"/>
-      <c r="P15" s="40"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+      <c r="O15" s="27"/>
+      <c r="P15" s="27"/>
       <c r="Q15" s="19"/>
       <c r="R15" s="19"/>
       <c r="S15" s="19"/>
@@ -5547,21 +5483,21 @@
       <c r="A16" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="40"/>
-      <c r="C16" s="40"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="40"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="40"/>
-      <c r="K16" s="40"/>
-      <c r="L16" s="40"/>
-      <c r="M16" s="40"/>
-      <c r="N16" s="40"/>
-      <c r="O16" s="40"/>
-      <c r="P16" s="40"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="27"/>
+      <c r="O16" s="27"/>
+      <c r="P16" s="27"/>
       <c r="Q16" s="19"/>
       <c r="R16" s="19"/>
       <c r="S16" s="19"/>
@@ -5570,21 +5506,21 @@
       <c r="A17" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="40"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="40"/>
-      <c r="I17" s="40"/>
-      <c r="J17" s="40"/>
-      <c r="K17" s="40"/>
-      <c r="L17" s="40"/>
-      <c r="M17" s="40"/>
-      <c r="N17" s="40"/>
-      <c r="O17" s="40"/>
-      <c r="P17" s="40"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="27"/>
+      <c r="L17" s="27"/>
+      <c r="M17" s="27"/>
+      <c r="N17" s="27"/>
+      <c r="O17" s="27"/>
+      <c r="P17" s="27"/>
       <c r="Q17" s="19"/>
       <c r="R17" s="19"/>
       <c r="S17" s="19"/>
@@ -5593,21 +5529,21 @@
       <c r="A18" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="40"/>
-      <c r="J18" s="40"/>
-      <c r="K18" s="40"/>
-      <c r="L18" s="40"/>
-      <c r="M18" s="40"/>
-      <c r="N18" s="40"/>
-      <c r="O18" s="40"/>
-      <c r="P18" s="40"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="27"/>
+      <c r="M18" s="27"/>
+      <c r="N18" s="27"/>
+      <c r="O18" s="27"/>
+      <c r="P18" s="27"/>
       <c r="Q18" s="19"/>
       <c r="R18" s="19"/>
       <c r="S18" s="19"/>
@@ -5616,21 +5552,21 @@
       <c r="A19" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="40"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="40"/>
-      <c r="J19" s="40"/>
-      <c r="K19" s="40"/>
-      <c r="L19" s="40"/>
-      <c r="M19" s="40"/>
-      <c r="N19" s="40"/>
-      <c r="O19" s="40"/>
-      <c r="P19" s="40"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="27"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27"/>
       <c r="Q19" s="19"/>
       <c r="R19" s="19"/>
       <c r="S19" s="19"/>
@@ -5639,21 +5575,21 @@
       <c r="A20" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="40"/>
-      <c r="C20" s="40"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="40"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="40"/>
-      <c r="J20" s="40"/>
-      <c r="K20" s="40"/>
-      <c r="L20" s="40"/>
-      <c r="M20" s="40"/>
-      <c r="N20" s="40"/>
-      <c r="O20" s="40"/>
-      <c r="P20" s="40"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="27"/>
+      <c r="N20" s="27"/>
+      <c r="O20" s="27"/>
+      <c r="P20" s="27"/>
       <c r="Q20" s="19"/>
       <c r="R20" s="19"/>
       <c r="S20" s="19"/>
@@ -5662,21 +5598,21 @@
       <c r="A21" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="40"/>
-      <c r="J21" s="40"/>
-      <c r="K21" s="40"/>
-      <c r="L21" s="40"/>
-      <c r="M21" s="40"/>
-      <c r="N21" s="40"/>
-      <c r="O21" s="40"/>
-      <c r="P21" s="40"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="27"/>
+      <c r="P21" s="27"/>
       <c r="Q21" s="19"/>
       <c r="R21" s="19"/>
       <c r="S21" s="19"/>
@@ -5685,21 +5621,21 @@
       <c r="A22" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="40"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="40"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="40"/>
-      <c r="J22" s="40"/>
-      <c r="K22" s="40"/>
-      <c r="L22" s="40"/>
-      <c r="M22" s="40"/>
-      <c r="N22" s="40"/>
-      <c r="O22" s="40"/>
-      <c r="P22" s="40"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
+      <c r="J22" s="27"/>
+      <c r="K22" s="27"/>
+      <c r="L22" s="27"/>
+      <c r="M22" s="27"/>
+      <c r="N22" s="27"/>
+      <c r="O22" s="27"/>
+      <c r="P22" s="27"/>
       <c r="Q22" s="19"/>
       <c r="R22" s="19"/>
       <c r="S22" s="19"/>
@@ -5708,21 +5644,21 @@
       <c r="A23" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B23" s="40"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="40"/>
-      <c r="J23" s="40"/>
-      <c r="K23" s="40"/>
-      <c r="L23" s="40"/>
-      <c r="M23" s="40"/>
-      <c r="N23" s="40"/>
-      <c r="O23" s="40"/>
-      <c r="P23" s="40"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
+      <c r="J23" s="27"/>
+      <c r="K23" s="27"/>
+      <c r="L23" s="27"/>
+      <c r="M23" s="27"/>
+      <c r="N23" s="27"/>
+      <c r="O23" s="27"/>
+      <c r="P23" s="27"/>
       <c r="Q23" s="19"/>
       <c r="R23" s="19"/>
       <c r="S23" s="19"/>
@@ -5731,21 +5667,21 @@
       <c r="A24" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="40"/>
-      <c r="C24" s="40"/>
-      <c r="D24" s="40"/>
-      <c r="E24" s="40"/>
-      <c r="F24" s="40"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="40"/>
-      <c r="J24" s="40"/>
-      <c r="K24" s="40"/>
-      <c r="L24" s="40"/>
-      <c r="M24" s="40"/>
-      <c r="N24" s="40"/>
-      <c r="O24" s="40"/>
-      <c r="P24" s="40"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
       <c r="Q24" s="19"/>
       <c r="R24" s="19"/>
       <c r="S24" s="19"/>
@@ -5754,21 +5690,21 @@
       <c r="A25" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="40"/>
-      <c r="C25" s="40"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="40"/>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="40"/>
-      <c r="J25" s="40"/>
-      <c r="K25" s="40"/>
-      <c r="L25" s="40"/>
-      <c r="M25" s="40"/>
-      <c r="N25" s="40"/>
-      <c r="O25" s="40"/>
-      <c r="P25" s="40"/>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
+      <c r="I25" s="27"/>
+      <c r="J25" s="27"/>
+      <c r="K25" s="27"/>
+      <c r="L25" s="27"/>
+      <c r="M25" s="27"/>
+      <c r="N25" s="27"/>
+      <c r="O25" s="27"/>
+      <c r="P25" s="27"/>
       <c r="Q25" s="19"/>
       <c r="R25" s="19"/>
       <c r="S25" s="19"/>
@@ -5796,7 +5732,7 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B27" s="21"/>
       <c r="C27" s="21"/>
@@ -5819,7 +5755,7 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="22" t="s">
-        <v>47</v>
+        <v>86</v>
       </c>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -5840,7 +5776,7 @@
       <c r="R28" s="22"/>
       <c r="S28" s="22"/>
     </row>
-    <row r="29" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="19"/>
       <c r="B29" s="19"/>
       <c r="C29" s="19"/>
@@ -5862,33 +5798,33 @@
       <c r="S29" s="19"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A30" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="B30" s="39"/>
-      <c r="C30" s="39"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="39"/>
-      <c r="H30" s="39"/>
-      <c r="I30" s="39"/>
-      <c r="J30" s="39"/>
-      <c r="K30" s="39"/>
-      <c r="L30" s="39"/>
-      <c r="M30" s="39"/>
-      <c r="N30" s="39"/>
-      <c r="O30" s="39"/>
-      <c r="P30" s="39"/>
-      <c r="Q30" s="39"/>
-      <c r="R30" s="39"/>
-      <c r="S30" s="39"/>
+      <c r="A30" s="42" t="s">
+        <v>87</v>
+      </c>
+      <c r="B30" s="42"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="42"/>
+      <c r="E30" s="42"/>
+      <c r="F30" s="42"/>
+      <c r="G30" s="42"/>
+      <c r="H30" s="42"/>
+      <c r="I30" s="42"/>
+      <c r="J30" s="42"/>
+      <c r="K30" s="42"/>
+      <c r="L30" s="42"/>
+      <c r="M30" s="42"/>
+      <c r="N30" s="42"/>
+      <c r="O30" s="42"/>
+      <c r="P30" s="42"/>
+      <c r="Q30" s="42"/>
+      <c r="R30" s="42"/>
+      <c r="S30" s="42"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="B31" s="40"/>
+        <v>88</v>
+      </c>
+      <c r="B31" s="27"/>
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
       <c r="E31" s="19"/>
@@ -5909,9 +5845,9 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="B32" s="40"/>
+        <v>89</v>
+      </c>
+      <c r="B32" s="27"/>
       <c r="C32" s="19"/>
       <c r="D32" s="19"/>
       <c r="E32" s="19"/>
@@ -5932,9 +5868,9 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>86</v>
-      </c>
-      <c r="B33" s="40"/>
+        <v>84</v>
+      </c>
+      <c r="B33" s="27"/>
       <c r="C33" s="19"/>
       <c r="D33" s="19"/>
       <c r="E33" s="19"/>
@@ -5953,7 +5889,7 @@
       <c r="R33" s="19"/>
       <c r="S33" s="19"/>
     </row>
-    <row r="34" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="19"/>
       <c r="B34" s="19"/>
       <c r="C34" s="19"/>
@@ -5976,16 +5912,16 @@
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B35" s="20" t="s">
+      <c r="C35" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="D35" s="20" t="s">
         <v>92</v>
-      </c>
-      <c r="C35" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="D35" s="20" t="s">
-        <v>93</v>
       </c>
       <c r="E35" s="20"/>
       <c r="F35" s="19"/>
@@ -6128,74 +6064,74 @@
   <sheetData>
     <row r="1" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="24" t="s">
         <v>94</v>
-      </c>
-      <c r="B1" s="24" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="24" t="s">
         <v>96</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>98</v>
-      </c>
-      <c r="B3" s="24" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" s="24" t="s">
         <v>100</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="24" t="s">
         <v>102</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="24" t="s">
         <v>104</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="24" t="s">
         <v>106</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" s="24" t="s">
         <v>108</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="B9" s="26" t="s">
         <v>110</v>
-      </c>
-      <c r="B9" s="26" t="s">
-        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>